<commit_message>
Integrate Axon reporting API with incremental cloud refresh
</commit_message>
<xml_diff>
--- a/automation/report-template.xlsx
+++ b/automation/report-template.xlsx
@@ -16,11 +16,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Quality" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Uncategorized'!$A$1:$X$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Uncategorized'!$A$1:$Y$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'AOR Summary'!$A$1:$K$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Component Summary'!$A$1:$K$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Owner Summary'!$A$1:$P$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Snapshot'!$A$1:$O$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Snapshot'!$A$1:$T$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Data Quality'!$A$1:$D$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -148,9 +148,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Uncategorized" displayName="Uncategorized" ref="A1:X1" headerRowCount="1">
-  <autoFilter ref="A1:X1"/>
-  <tableColumns count="24">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Uncategorized" displayName="Uncategorized" ref="A1:Y1" headerRowCount="1">
+  <autoFilter ref="A1:Y1"/>
+  <tableColumns count="25">
     <tableColumn id="1" name="Run ID"/>
     <tableColumn id="2" name="Snapshot Date"/>
     <tableColumn id="3" name="Fiscal Year"/>
@@ -175,6 +175,7 @@
     <tableColumn id="22" name="Component Name"/>
     <tableColumn id="23" name="AOR"/>
     <tableColumn id="24" name="Data Quality Notes"/>
+    <tableColumn id="25" name="External Evidence ID"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -246,9 +247,9 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Snapshot" displayName="Snapshot" ref="A1:O2" headerRowCount="1">
-  <autoFilter ref="A1:O2"/>
-  <tableColumns count="15">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Snapshot" displayName="Snapshot" ref="A1:T2" headerRowCount="1">
+  <autoFilter ref="A1:T2"/>
+  <tableColumns count="20">
     <tableColumn id="1" name="Run ID"/>
     <tableColumn id="2" name="Snapshot Date"/>
     <tableColumn id="3" name="Fiscal Year"/>
@@ -264,6 +265,11 @@
     <tableColumn id="13" name="Excluded Status Rows"/>
     <tableColumn id="14" name="Categorized Rows"/>
     <tableColumn id="15" name="Rejected Rows"/>
+    <tableColumn id="16" name="Sample Data"/>
+    <tableColumn id="17" name="Source Data Date"/>
+    <tableColumn id="18" name="Source Report"/>
+    <tableColumn id="19" name="Creation From Date"/>
+    <tableColumn id="20" name="Creation To Date"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -651,7 +657,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1"/>
+  <dimension ref="A1:Y1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -678,6 +684,7 @@
     <col width="16" customWidth="1" min="22" max="22"/>
     <col width="14" customWidth="1" min="23" max="23"/>
     <col width="20" customWidth="1" min="24" max="24"/>
+    <col width="22" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -801,9 +808,14 @@
           <t>Data Quality Notes</t>
         </is>
       </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>External Evidence ID</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:X1"/>
+  <autoFilter ref="A1:Y1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -1111,7 +1123,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:T2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1129,6 +1141,11 @@
     <col width="22" customWidth="1" min="13" max="13"/>
     <col width="18" customWidth="1" min="14" max="14"/>
     <col width="15" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="17" max="17"/>
+    <col width="15" customWidth="1" min="18" max="18"/>
+    <col width="20" customWidth="1" min="19" max="19"/>
+    <col width="18" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1207,6 +1224,31 @@
           <t>Rejected Rows</t>
         </is>
       </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Sample Data</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Source Data Date</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Source Report</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Creation From Date</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>Creation To Date</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1258,9 +1300,20 @@
       <c r="O2" t="n">
         <v>0</v>
       </c>
+      <c r="P2" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>CSV export</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O2"/>
+  <autoFilter ref="A1:T2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>